<commit_message>
Update calibration scripts and workbook to include StopFrequency
Minor Adjustment to tour_mode_choice scripts and TripModeChoice workbook
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/12_StopFrequency_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/12_StopFrequency_2023_blank.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30678C82-A27B-4E2F-BBCC-34F5F4A83B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EFF5F0-9AF8-4ED4-B943-FD306474D47C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1191E293-BD99-4EAF-97FD-32238A032A8E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1191E293-BD99-4EAF-97FD-32238A032A8E}"/>
   </bookViews>
   <sheets>
     <sheet name="calibration" sheetId="2" r:id="rId1"/>
-    <sheet name="modeldata" sheetId="1" r:id="rId2"/>
-    <sheet name="BATS 2023" sheetId="3" r:id="rId3"/>
+    <sheet name="constants" sheetId="4" r:id="rId2"/>
+    <sheet name="modeldata" sheetId="1" r:id="rId3"/>
+    <sheet name="BATS 2023" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,8 +41,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="88">
   <si>
     <t>Source:</t>
   </si>
@@ -231,6 +254,81 @@
   <si>
     <t>4+ out 4+ ret</t>
   </si>
+  <si>
+    <t>Alt1</t>
+  </si>
+  <si>
+    <t>Alt2</t>
+  </si>
+  <si>
+    <t>Alt3</t>
+  </si>
+  <si>
+    <t>Alt4</t>
+  </si>
+  <si>
+    <t>Alt5</t>
+  </si>
+  <si>
+    <t>Alt6</t>
+  </si>
+  <si>
+    <t>Alt7</t>
+  </si>
+  <si>
+    <t>Alt8</t>
+  </si>
+  <si>
+    <t>Alt9</t>
+  </si>
+  <si>
+    <t>Alt10</t>
+  </si>
+  <si>
+    <t>Alt11</t>
+  </si>
+  <si>
+    <t>Alt12</t>
+  </si>
+  <si>
+    <t>Alt13</t>
+  </si>
+  <si>
+    <t>Alt14</t>
+  </si>
+  <si>
+    <t>Alt15</t>
+  </si>
+  <si>
+    <t>Alt16</t>
+  </si>
+  <si>
+    <t>4 Stops</t>
+  </si>
+  <si>
+    <t>5 Stops</t>
+  </si>
+  <si>
+    <t>2 out</t>
+  </si>
+  <si>
+    <t>Return Stops</t>
+  </si>
+  <si>
+    <t>Total Number of Stops</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Exisiting</t>
+  </si>
+  <si>
+    <t>New Constants</t>
+  </si>
+  <si>
+    <t>Outbound Stops</t>
+  </si>
 </sst>
 </file>
 
@@ -241,7 +339,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,6 +377,14 @@
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -413,7 +519,7 @@
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -493,13 +599,27 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -6404,7 +6524,7 @@
       </c>
       <c r="C48" s="11"/>
     </row>
-    <row r="50" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>51</v>
       </c>
@@ -6415,7 +6535,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="51" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:39" x14ac:dyDescent="0.25">
       <c r="C51" t="s">
         <v>1</v>
       </c>
@@ -6516,21 +6636,57 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>87</v>
+      </c>
       <c r="B52" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C52" s="16"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="17"/>
-      <c r="F52" s="17"/>
-      <c r="G52" s="17"/>
-      <c r="H52" s="17"/>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
-      <c r="M52" s="18"/>
+      <c r="C52" s="16" cm="1">
+        <f t="array" ref="C52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="17" cm="1">
+        <f t="array" ref="D52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="17" cm="1">
+        <f t="array" ref="E52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="17" cm="1">
+        <f t="array" ref="F52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G52" s="17" cm="1">
+        <f t="array" ref="G52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="17" cm="1">
+        <f t="array" ref="H52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I52" s="17" cm="1">
+        <f t="array" ref="I52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J52" s="17" cm="1">
+        <f t="array" ref="J52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K52" s="17" cm="1">
+        <f t="array" ref="K52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L52" s="17" cm="1">
+        <f t="array" ref="L52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M52" s="18" cm="1">
+        <f t="array" ref="M52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
       <c r="O52" s="15" t="s">
         <v>33</v>
       </c>
@@ -6593,21 +6749,57 @@
       <c r="AL52" s="17"/>
       <c r="AM52" s="18"/>
     </row>
-    <row r="53" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>87</v>
+      </c>
       <c r="B53" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C53" s="19"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="15"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="20"/>
+      <c r="C53" s="19" cm="1">
+        <f t="array" ref="C53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D53" s="15" cm="1">
+        <f t="array" ref="D53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="15" cm="1">
+        <f t="array" ref="E53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="15" cm="1">
+        <f t="array" ref="F53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G53" s="15" cm="1">
+        <f t="array" ref="G53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H53" s="15" cm="1">
+        <f t="array" ref="H53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="15" cm="1">
+        <f t="array" ref="I53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J53" s="15" cm="1">
+        <f t="array" ref="J53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K53" s="15" cm="1">
+        <f t="array" ref="K53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L53" s="15" cm="1">
+        <f t="array" ref="L53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M53" s="20" cm="1">
+        <f t="array" ref="M53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
       <c r="O53" s="15" t="s">
         <v>34</v>
       </c>
@@ -6703,21 +6895,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="54" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>87</v>
+      </c>
       <c r="B54" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C54" s="19"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="15"/>
-      <c r="F54" s="15"/>
-      <c r="G54" s="15"/>
-      <c r="H54" s="15"/>
-      <c r="I54" s="15"/>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="20"/>
+      <c r="C54" s="19" cm="1">
+        <f t="array" ref="C54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="15" cm="1">
+        <f t="array" ref="D54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E54" s="15" cm="1">
+        <f t="array" ref="E54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F54" s="15" cm="1">
+        <f t="array" ref="F54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G54" s="15" cm="1">
+        <f t="array" ref="G54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H54" s="15" cm="1">
+        <f t="array" ref="H54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="15" cm="1">
+        <f t="array" ref="I54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J54" s="15" cm="1">
+        <f t="array" ref="J54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K54" s="15" cm="1">
+        <f t="array" ref="K54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L54" s="15" cm="1">
+        <f t="array" ref="L54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M54" s="20" cm="1">
+        <f t="array" ref="M54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
       <c r="O54" s="15" t="s">
         <v>35</v>
       </c>
@@ -6813,21 +7041,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="55" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>87</v>
+      </c>
       <c r="B55" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C55" s="21"/>
-      <c r="D55" s="22"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-      <c r="G55" s="22"/>
-      <c r="H55" s="22"/>
-      <c r="I55" s="22"/>
-      <c r="J55" s="22"/>
-      <c r="K55" s="22"/>
-      <c r="L55" s="22"/>
-      <c r="M55" s="23"/>
+      <c r="C55" s="21" cm="1">
+        <f t="array" ref="C55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D55" s="22" cm="1">
+        <f t="array" ref="D55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E55" s="22" cm="1">
+        <f t="array" ref="E55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="22" cm="1">
+        <f t="array" ref="F55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="22" cm="1">
+        <f t="array" ref="G55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H55" s="22" cm="1">
+        <f t="array" ref="H55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="22" cm="1">
+        <f t="array" ref="I55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="22" cm="1">
+        <f t="array" ref="J55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K55" s="22" cm="1">
+        <f t="array" ref="K55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L55" s="22" cm="1">
+        <f t="array" ref="L55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M55" s="23" cm="1">
+        <f t="array" ref="M55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
+        <v>0</v>
+      </c>
       <c r="O55" s="15" t="s">
         <v>36</v>
       </c>
@@ -6923,21 +7187,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="56" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>82</v>
+      </c>
       <c r="B56" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C56" s="24"/>
-      <c r="D56" s="25"/>
-      <c r="E56" s="25"/>
-      <c r="F56" s="25"/>
-      <c r="G56" s="25"/>
-      <c r="H56" s="25"/>
-      <c r="I56" s="25"/>
-      <c r="J56" s="25"/>
-      <c r="K56" s="25"/>
-      <c r="L56" s="25"/>
-      <c r="M56" s="26"/>
+      <c r="C56" s="24" cm="1">
+        <f t="array" ref="C56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D56" s="25" cm="1">
+        <f t="array" ref="D56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E56" s="25" cm="1">
+        <f t="array" ref="E56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F56" s="25" cm="1">
+        <f t="array" ref="F56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G56" s="25" cm="1">
+        <f t="array" ref="G56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H56" s="25" cm="1">
+        <f t="array" ref="H56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I56" s="25" cm="1">
+        <f t="array" ref="I56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J56" s="25" cm="1">
+        <f t="array" ref="J56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K56" s="25" cm="1">
+        <f t="array" ref="K56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L56" s="25" cm="1">
+        <f t="array" ref="L56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M56" s="26" cm="1">
+        <f t="array" ref="M56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
       <c r="O56" s="13" t="s">
         <v>29</v>
       </c>
@@ -7000,21 +7300,57 @@
       <c r="AL56" s="25"/>
       <c r="AM56" s="26"/>
     </row>
-    <row r="57" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>82</v>
+      </c>
       <c r="B57" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C57" s="27"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="13"/>
-      <c r="H57" s="13"/>
-      <c r="I57" s="13"/>
-      <c r="J57" s="13"/>
-      <c r="K57" s="13"/>
-      <c r="L57" s="13"/>
-      <c r="M57" s="28"/>
+      <c r="C57" s="27" cm="1">
+        <f t="array" ref="C57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D57" s="13" cm="1">
+        <f t="array" ref="D57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E57" s="13" cm="1">
+        <f t="array" ref="E57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F57" s="13" cm="1">
+        <f t="array" ref="F57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G57" s="13" cm="1">
+        <f t="array" ref="G57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="13" cm="1">
+        <f t="array" ref="H57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I57" s="13" cm="1">
+        <f t="array" ref="I57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J57" s="13" cm="1">
+        <f t="array" ref="J57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K57" s="13" cm="1">
+        <f t="array" ref="K57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L57" s="13" cm="1">
+        <f t="array" ref="L57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M57" s="28" cm="1">
+        <f t="array" ref="M57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
       <c r="O57" s="13" t="s">
         <v>30</v>
       </c>
@@ -7110,21 +7446,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="58" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>82</v>
+      </c>
       <c r="B58" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C58" s="27"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="13"/>
-      <c r="G58" s="13"/>
-      <c r="H58" s="13"/>
-      <c r="I58" s="13"/>
-      <c r="J58" s="13"/>
-      <c r="K58" s="13"/>
-      <c r="L58" s="13"/>
-      <c r="M58" s="28"/>
+      <c r="C58" s="27" cm="1">
+        <f t="array" ref="C58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D58" s="13" cm="1">
+        <f t="array" ref="D58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E58" s="13" cm="1">
+        <f t="array" ref="E58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="13" cm="1">
+        <f t="array" ref="F58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G58" s="13" cm="1">
+        <f t="array" ref="G58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H58" s="13" cm="1">
+        <f t="array" ref="H58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I58" s="13" cm="1">
+        <f t="array" ref="I58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J58" s="13" cm="1">
+        <f t="array" ref="J58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K58" s="13" cm="1">
+        <f t="array" ref="K58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L58" s="13" cm="1">
+        <f t="array" ref="L58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M58" s="28" cm="1">
+        <f t="array" ref="M58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
       <c r="O58" s="13" t="s">
         <v>31</v>
       </c>
@@ -7220,21 +7592,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="59" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>82</v>
+      </c>
       <c r="B59" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="C59" s="29"/>
-      <c r="D59" s="30"/>
-      <c r="E59" s="30"/>
-      <c r="F59" s="30"/>
-      <c r="G59" s="30"/>
-      <c r="H59" s="30"/>
-      <c r="I59" s="30"/>
-      <c r="J59" s="30"/>
-      <c r="K59" s="30"/>
-      <c r="L59" s="30"/>
-      <c r="M59" s="31"/>
+      <c r="C59" s="29" cm="1">
+        <f t="array" ref="C59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D59" s="30" cm="1">
+        <f t="array" ref="D59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E59" s="30" cm="1">
+        <f t="array" ref="E59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="30" cm="1">
+        <f t="array" ref="F59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G59" s="30" cm="1">
+        <f t="array" ref="G59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H59" s="30" cm="1">
+        <f t="array" ref="H59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I59" s="30" cm="1">
+        <f t="array" ref="I59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J59" s="30" cm="1">
+        <f t="array" ref="J59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K59" s="30" cm="1">
+        <f t="array" ref="K59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L59" s="30" cm="1">
+        <f t="array" ref="L59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M59" s="31" cm="1">
+        <f t="array" ref="M59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
+        <v>0</v>
+      </c>
       <c r="O59" s="13" t="s">
         <v>32</v>
       </c>
@@ -7330,21 +7738,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="60" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>83</v>
+      </c>
       <c r="B60" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C60" s="32"/>
-      <c r="D60" s="33"/>
-      <c r="E60" s="33"/>
-      <c r="F60" s="33"/>
-      <c r="G60" s="33"/>
-      <c r="H60" s="33"/>
-      <c r="I60" s="33"/>
-      <c r="J60" s="33"/>
-      <c r="K60" s="33"/>
-      <c r="L60" s="33"/>
-      <c r="M60" s="34"/>
+      <c r="C60" s="32" cm="1">
+        <f t="array" ref="C60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D60" s="33" cm="1">
+        <f t="array" ref="D60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E60" s="33" cm="1">
+        <f t="array" ref="E60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F60" s="33" cm="1">
+        <f t="array" ref="F60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G60" s="33" cm="1">
+        <f t="array" ref="G60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H60" s="33" cm="1">
+        <f t="array" ref="H60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I60" s="33" cm="1">
+        <f t="array" ref="I60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J60" s="33" cm="1">
+        <f t="array" ref="J60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K60" s="33" cm="1">
+        <f t="array" ref="K60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L60" s="33" cm="1">
+        <f t="array" ref="L60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M60" s="34" cm="1">
+        <f t="array" ref="M60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O60" s="14" t="s">
         <v>43</v>
       </c>
@@ -7407,21 +7851,57 @@
       <c r="AL60" s="33"/>
       <c r="AM60" s="34"/>
     </row>
-    <row r="61" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>83</v>
+      </c>
       <c r="B61" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="C61" s="35"/>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="14"/>
-      <c r="I61" s="14"/>
-      <c r="J61" s="14"/>
-      <c r="K61" s="14"/>
-      <c r="L61" s="14"/>
-      <c r="M61" s="36"/>
+      <c r="C61" s="35" cm="1">
+        <f t="array" ref="C61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="14" cm="1">
+        <f t="array" ref="D61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E61" s="14" cm="1">
+        <f t="array" ref="E61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F61" s="14" cm="1">
+        <f t="array" ref="F61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G61" s="14" cm="1">
+        <f t="array" ref="G61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H61" s="14" cm="1">
+        <f t="array" ref="H61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I61" s="14" cm="1">
+        <f t="array" ref="I61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J61" s="14" cm="1">
+        <f t="array" ref="J61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K61" s="14" cm="1">
+        <f t="array" ref="K61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L61" s="14" cm="1">
+        <f t="array" ref="L61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M61" s="36" cm="1">
+        <f t="array" ref="M61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O61" s="14" t="s">
         <v>37</v>
       </c>
@@ -7484,21 +7964,57 @@
       <c r="AL61" s="14"/>
       <c r="AM61" s="36"/>
     </row>
-    <row r="62" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>83</v>
+      </c>
       <c r="B62" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C62" s="35"/>
-      <c r="D62" s="14"/>
-      <c r="E62" s="14"/>
-      <c r="F62" s="14"/>
-      <c r="G62" s="14"/>
-      <c r="H62" s="14"/>
-      <c r="I62" s="14"/>
-      <c r="J62" s="14"/>
-      <c r="K62" s="14"/>
-      <c r="L62" s="14"/>
-      <c r="M62" s="36"/>
+      <c r="C62" s="35" cm="1">
+        <f t="array" ref="C62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="14" cm="1">
+        <f t="array" ref="D62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E62" s="14" cm="1">
+        <f t="array" ref="E62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F62" s="14" cm="1">
+        <f t="array" ref="F62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G62" s="14" cm="1">
+        <f t="array" ref="G62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H62" s="14" cm="1">
+        <f t="array" ref="H62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I62" s="14" cm="1">
+        <f t="array" ref="I62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J62" s="14" cm="1">
+        <f t="array" ref="J62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K62" s="14" cm="1">
+        <f t="array" ref="K62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L62" s="14" cm="1">
+        <f t="array" ref="L62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M62" s="36" cm="1">
+        <f t="array" ref="M62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O62" s="14" t="s">
         <v>38</v>
       </c>
@@ -7594,21 +8110,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="63" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>83</v>
+      </c>
       <c r="B63" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C63" s="35"/>
-      <c r="D63" s="14"/>
-      <c r="E63" s="14"/>
-      <c r="F63" s="14"/>
-      <c r="G63" s="14"/>
-      <c r="H63" s="14"/>
-      <c r="I63" s="14"/>
-      <c r="J63" s="14"/>
-      <c r="K63" s="14"/>
-      <c r="L63" s="14"/>
-      <c r="M63" s="36"/>
+      <c r="C63" s="35" cm="1">
+        <f t="array" ref="C63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D63" s="14" cm="1">
+        <f t="array" ref="D63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E63" s="14" cm="1">
+        <f t="array" ref="E63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F63" s="14" cm="1">
+        <f t="array" ref="F63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G63" s="14" cm="1">
+        <f t="array" ref="G63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H63" s="14" cm="1">
+        <f t="array" ref="H63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I63" s="14" cm="1">
+        <f t="array" ref="I63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J63" s="14" cm="1">
+        <f t="array" ref="J63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K63" s="14" cm="1">
+        <f t="array" ref="K63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L63" s="14" cm="1">
+        <f t="array" ref="L63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M63" s="36" cm="1">
+        <f t="array" ref="M63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O63" s="14" t="s">
         <v>39</v>
       </c>
@@ -7704,21 +8256,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="64" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>83</v>
+      </c>
       <c r="B64" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="C64" s="35"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="14"/>
-      <c r="J64" s="14"/>
-      <c r="K64" s="14"/>
-      <c r="L64" s="14"/>
-      <c r="M64" s="36"/>
+        <v>79</v>
+      </c>
+      <c r="C64" s="35" cm="1">
+        <f t="array" ref="C64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D64" s="14" cm="1">
+        <f t="array" ref="D64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E64" s="14" cm="1">
+        <f t="array" ref="E64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F64" s="14" cm="1">
+        <f t="array" ref="F64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G64" s="14" cm="1">
+        <f t="array" ref="G64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H64" s="14" cm="1">
+        <f t="array" ref="H64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I64" s="14" cm="1">
+        <f t="array" ref="I64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J64" s="14" cm="1">
+        <f t="array" ref="J64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K64" s="14" cm="1">
+        <f t="array" ref="K64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L64" s="14" cm="1">
+        <f t="array" ref="L64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M64" s="36" cm="1">
+        <f t="array" ref="M64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O64" s="14" t="s">
         <v>44</v>
       </c>
@@ -7767,7 +8355,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB64" s="14" t="s">
-        <v>44</v>
+        <v>79</v>
       </c>
       <c r="AC64" s="35" t="e">
         <f t="shared" si="185"/>
@@ -7814,21 +8402,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="65" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>83</v>
+      </c>
       <c r="B65" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C65" s="35"/>
-      <c r="D65" s="14"/>
-      <c r="E65" s="14"/>
-      <c r="F65" s="14"/>
-      <c r="G65" s="14"/>
-      <c r="H65" s="14"/>
-      <c r="I65" s="14"/>
-      <c r="J65" s="14"/>
-      <c r="K65" s="14"/>
-      <c r="L65" s="14"/>
-      <c r="M65" s="36"/>
+        <v>80</v>
+      </c>
+      <c r="C65" s="35" cm="1">
+        <f t="array" ref="C65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D65" s="14" cm="1">
+        <f t="array" ref="D65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E65" s="14" cm="1">
+        <f t="array" ref="E65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F65" s="14" cm="1">
+        <f t="array" ref="F65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G65" s="14" cm="1">
+        <f t="array" ref="G65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H65" s="14" cm="1">
+        <f t="array" ref="H65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I65" s="14" cm="1">
+        <f t="array" ref="I65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J65" s="14" cm="1">
+        <f t="array" ref="J65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K65" s="14" cm="1">
+        <f t="array" ref="K65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L65" s="14" cm="1">
+        <f t="array" ref="L65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M65" s="36" cm="1">
+        <f t="array" ref="M65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O65" s="14" t="s">
         <v>45</v>
       </c>
@@ -7877,7 +8501,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB65" s="14" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="AC65" s="35" t="e">
         <f t="shared" si="185"/>
@@ -7924,21 +8548,57 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="66" spans="2:39" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>83</v>
+      </c>
       <c r="B66" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C66" s="37"/>
-      <c r="D66" s="38"/>
-      <c r="E66" s="38"/>
-      <c r="F66" s="38"/>
-      <c r="G66" s="38"/>
-      <c r="H66" s="38"/>
-      <c r="I66" s="38"/>
-      <c r="J66" s="38"/>
-      <c r="K66" s="38"/>
-      <c r="L66" s="38"/>
-      <c r="M66" s="39"/>
+      <c r="C66" s="37" cm="1">
+        <f t="array" ref="C66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="38" cm="1">
+        <f t="array" ref="D66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!D$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="E66" s="38" cm="1">
+        <f t="array" ref="E66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!E$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="F66" s="38" cm="1">
+        <f t="array" ref="F66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!F$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="G66" s="38" cm="1">
+        <f t="array" ref="G66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!G$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="38" cm="1">
+        <f t="array" ref="H66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!H$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I66" s="38" cm="1">
+        <f t="array" ref="I66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!I$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J66" s="38" cm="1">
+        <f t="array" ref="J66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!J$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="K66" s="38" cm="1">
+        <f t="array" ref="K66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!K$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="L66" s="38" cm="1">
+        <f t="array" ref="L66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!L$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
+      <c r="M66" s="39" cm="1">
+        <f t="array" ref="M66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!M$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
+        <v>0</v>
+      </c>
       <c r="O66" s="14" t="s">
         <v>40</v>
       </c>
@@ -8031,6 +8691,2836 @@
       </c>
       <c r="AM66" s="39" t="e">
         <f t="shared" si="195"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="AC27:AM45">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>ABS(AC27) &gt; 10%</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F41A67D-DB7F-48D1-AFB6-344D1665DF25}">
+  <dimension ref="A1:AH38"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="20.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="C1" s="73" t="s">
+        <v>85</v>
+      </c>
+      <c r="S1" s="73" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+      <c r="J2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K2" t="s">
+        <v>71</v>
+      </c>
+      <c r="L2" t="s">
+        <v>72</v>
+      </c>
+      <c r="M2" t="s">
+        <v>73</v>
+      </c>
+      <c r="N2" t="s">
+        <v>74</v>
+      </c>
+      <c r="O2" t="s">
+        <v>75</v>
+      </c>
+      <c r="P2" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>77</v>
+      </c>
+      <c r="R2" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="S2" t="s">
+        <v>63</v>
+      </c>
+      <c r="T2" t="s">
+        <v>64</v>
+      </c>
+      <c r="U2" t="s">
+        <v>65</v>
+      </c>
+      <c r="V2" t="s">
+        <v>66</v>
+      </c>
+      <c r="W2" t="s">
+        <v>67</v>
+      </c>
+      <c r="X2" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>71</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>72</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>73</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>75</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>76</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L3" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s">
+        <v>79</v>
+      </c>
+      <c r="N3" t="s">
+        <v>80</v>
+      </c>
+      <c r="O3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>80</v>
+      </c>
+      <c r="R3" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="S3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" t="s">
+        <v>37</v>
+      </c>
+      <c r="U3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>37</v>
+      </c>
+      <c r="X3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
+        <v>81</v>
+      </c>
+      <c r="L4" t="s">
+        <v>81</v>
+      </c>
+      <c r="M4" t="s">
+        <v>81</v>
+      </c>
+      <c r="N4" t="s">
+        <v>81</v>
+      </c>
+      <c r="O4" t="s">
+        <v>36</v>
+      </c>
+      <c r="P4" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>36</v>
+      </c>
+      <c r="R4" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S4" t="s">
+        <v>33</v>
+      </c>
+      <c r="T4" t="s">
+        <v>33</v>
+      </c>
+      <c r="U4" t="s">
+        <v>33</v>
+      </c>
+      <c r="V4" t="s">
+        <v>33</v>
+      </c>
+      <c r="W4" t="s">
+        <v>34</v>
+      </c>
+      <c r="X4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>81</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>81</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>81</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>81</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>36</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A5" s="73" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="R5" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="S5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="U5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="V5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="W5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="X5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Z5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="AA5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="AB5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="AD5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="AE5" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG5" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH5" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>87</v>
+      </c>
+      <c r="R6" s="7"/>
+      <c r="S6">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH6" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A6,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="R7" s="7"/>
+      <c r="S7">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W7">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA7">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE7">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH7" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A7,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>83</v>
+      </c>
+      <c r="R8" s="7"/>
+      <c r="S8">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W8">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH8" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A8,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>87</v>
+      </c>
+      <c r="R9" s="7"/>
+      <c r="S9">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH9" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A9,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>82</v>
+      </c>
+      <c r="R10" s="7"/>
+      <c r="S10">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W10">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA10">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE10">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH10" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A10,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" t="s">
+        <v>83</v>
+      </c>
+      <c r="R11" s="7"/>
+      <c r="S11">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W11">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH11" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A11,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>87</v>
+      </c>
+      <c r="R12" s="7"/>
+      <c r="S12">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH12" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A12,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>82</v>
+      </c>
+      <c r="R13" s="7"/>
+      <c r="S13">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W13">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA13">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE13">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH13" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A13,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>83</v>
+      </c>
+      <c r="R14" s="7"/>
+      <c r="S14">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W14">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH14" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A14,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" t="s">
+        <v>87</v>
+      </c>
+      <c r="R15" s="7"/>
+      <c r="S15">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH15" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A15,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" t="s">
+        <v>82</v>
+      </c>
+      <c r="R16" s="7"/>
+      <c r="S16">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W16">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA16">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE16">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH16" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A16,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" t="s">
+        <v>83</v>
+      </c>
+      <c r="R17" s="7"/>
+      <c r="S17">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W17">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH17" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A17,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" t="s">
+        <v>87</v>
+      </c>
+      <c r="R18" s="7"/>
+      <c r="S18">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH18" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A18,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" t="s">
+        <v>82</v>
+      </c>
+      <c r="R19" s="7"/>
+      <c r="S19">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W19">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA19">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE19">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH19" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A19,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" t="s">
+        <v>83</v>
+      </c>
+      <c r="R20" s="7"/>
+      <c r="S20">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W20">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH20" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A20,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" t="s">
+        <v>87</v>
+      </c>
+      <c r="R21" s="7"/>
+      <c r="S21">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V21">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH21" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A21,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" t="s">
+        <v>82</v>
+      </c>
+      <c r="R22" s="7"/>
+      <c r="S22">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W22">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA22">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE22">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH22" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A22,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" t="s">
+        <v>83</v>
+      </c>
+      <c r="R23" s="7"/>
+      <c r="S23">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W23">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH23" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A23,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>7</v>
+      </c>
+      <c r="B24" t="s">
+        <v>87</v>
+      </c>
+      <c r="R24" s="7"/>
+      <c r="S24">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V24">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH24" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A24,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B25" t="s">
+        <v>82</v>
+      </c>
+      <c r="R25" s="7"/>
+      <c r="S25">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W25">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA25">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE25">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH25" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A25,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" t="s">
+        <v>83</v>
+      </c>
+      <c r="R26" s="7"/>
+      <c r="S26">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W26">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH26" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A26,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27" t="s">
+        <v>87</v>
+      </c>
+      <c r="R27" s="7"/>
+      <c r="S27">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T27">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U27">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V27">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH27" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A27,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" t="s">
+        <v>82</v>
+      </c>
+      <c r="R28" s="7"/>
+      <c r="S28">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W28">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA28">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE28">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH28" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A28,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29" t="s">
+        <v>83</v>
+      </c>
+      <c r="R29" s="7"/>
+      <c r="S29">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W29">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH29" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A29,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" t="s">
+        <v>87</v>
+      </c>
+      <c r="R30" s="7"/>
+      <c r="S30">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U30">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V30">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH30" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A30,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s">
+        <v>82</v>
+      </c>
+      <c r="R31" s="7"/>
+      <c r="S31">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W31">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA31">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE31">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH31" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A31,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="32" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" t="s">
+        <v>83</v>
+      </c>
+      <c r="R32" s="7"/>
+      <c r="S32">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W32">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH32" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A32,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="33" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" t="s">
+        <v>87</v>
+      </c>
+      <c r="R33" s="7"/>
+      <c r="S33">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U33">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V33">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH33" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A33,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="34" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" t="s">
+        <v>82</v>
+      </c>
+      <c r="R34" s="7"/>
+      <c r="S34">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W34">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA34">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE34">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH34" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A34,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="35" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" t="s">
+        <v>83</v>
+      </c>
+      <c r="R35" s="7"/>
+      <c r="S35">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T35">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W35">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH35" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A35,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="36" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>11</v>
+      </c>
+      <c r="B36" t="s">
+        <v>87</v>
+      </c>
+      <c r="R36" s="7"/>
+      <c r="S36">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!S$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T36">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!T$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U36">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!U$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="V36">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!V$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="W36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!W$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="X36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!X$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Y$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!Z$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AA$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AB$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AC$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AD$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AE$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AF$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AG$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH36" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(constants!AH$4,calibration!$AB$52:$AB$66,0),MATCH(constants!$A36,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="37" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" t="s">
+        <v>82</v>
+      </c>
+      <c r="R37" s="7"/>
+      <c r="S37">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W37">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA37">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AB37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE37">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="AF37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH37" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$5,calibration!$AB$52:$AB$66,0),MATCH(constants!$A37,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="38" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" t="s">
+        <v>83</v>
+      </c>
+      <c r="R38" s="7"/>
+      <c r="S38">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(S$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="T38">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(T$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="U38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(U$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(V$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="W38">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(W$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>0</v>
+      </c>
+      <c r="X38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(X$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Y38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Y$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="Z38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(Z$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AA38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AA$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AB38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AB$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AC38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AC$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AD38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AD$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AE38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AE$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AF38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AF$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AG38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AG$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="AH38" t="e">
+        <f>INDEX(calibration!$AC$52:$AM$66,MATCH(AH$3,calibration!$AB$52:$AB$66,0),MATCH(constants!$A38,calibration!$P$51:$Z$51,0))</f>
         <v>#DIV/0!</v>
       </c>
     </row>
@@ -8039,7 +11529,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6ADE016D-553D-4789-A918-6381BA0F9838}">
   <sheetPr>
     <tabColor rgb="FF9BBB59"/>
@@ -8191,7 +11681,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAEE3413-48B7-4B37-B389-374873CCA87C}">
   <sheetPr>
     <tabColor theme="3" tint="0.499984740745262"/>

</xml_diff>

<commit_message>
Edit UEC script to correct mapping
Minor edits to StopFrequency and TripModeChoice calibration templates
</commit_message>
<xml_diff>
--- a/utilities/calibration/workbook_templates/12_StopFrequency_2023_blank.xlsx
+++ b/utilities/calibration/workbook_templates/12_StopFrequency_2023_blank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\travel-model-one\utilities\calibration\workbook_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82EFF5F0-9AF8-4ED4-B943-FD306474D47C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DECCF4F-D169-4FA8-9A53-E82CC1C9364E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1191E293-BD99-4EAF-97FD-32238A032A8E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1191E293-BD99-4EAF-97FD-32238A032A8E}"/>
   </bookViews>
   <sheets>
     <sheet name="calibration" sheetId="2" r:id="rId1"/>
@@ -148,9 +148,6 @@
   </si>
   <si>
     <t>3 out 3 ret</t>
-  </si>
-  <si>
-    <t>Source</t>
   </si>
   <si>
     <t>0 Ret</t>
@@ -328,6 +325,9 @@
   </si>
   <si>
     <t>Outbound Stops</t>
+  </si>
+  <si>
+    <t>Source: M:\Development\Travel Model One\Calibration\Version 1.7\2023_BATS_Summaries\pipeline_mt_20260821_NoMon_rmo\ctramp_2023\BATS_Summaries\BATS2023_stop_frequency.xlsx</t>
   </si>
 </sst>
 </file>
@@ -606,13 +606,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <strike val="0"/>
@@ -971,7 +965,7 @@
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
       <c r="C2" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D2" s="12"/>
       <c r="E2" s="12"/>
@@ -985,7 +979,7 @@
       <c r="M2" s="12"/>
       <c r="N2" s="12"/>
       <c r="O2" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
@@ -1000,7 +994,7 @@
       <c r="Z2" s="12"/>
       <c r="AA2" s="12"/>
       <c r="AB2" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AC2" s="12"/>
       <c r="AD2" s="12"/>
@@ -1117,7 +1111,7 @@
     </row>
     <row r="4" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" s="43">
         <f>SUM('BATS 2023'!P4:P7)</f>
@@ -1164,7 +1158,7 @@
         <v>856344.68628552498</v>
       </c>
       <c r="O4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P4" s="43">
         <f>SUM(modeldata!C4:C7)</f>
@@ -1211,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="AB4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AC4" s="3">
         <f>P4-C4</f>
@@ -1260,7 +1254,7 @@
     </row>
     <row r="5" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" s="46">
         <f>SUM('BATS 2023'!P8:P11)</f>
@@ -1307,7 +1301,7 @@
         <v>84280.883866961944</v>
       </c>
       <c r="O5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P5" s="46">
         <f>SUM(modeldata!C8:C11)</f>
@@ -1354,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="AB5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AC5" s="6">
         <f>P5-C5</f>
@@ -1403,7 +1397,7 @@
     </row>
     <row r="6" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" s="46">
         <f>SUM('BATS 2023'!P12:P15)</f>
@@ -1450,7 +1444,7 @@
         <v>37720.411891635027</v>
       </c>
       <c r="O6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P6" s="46">
         <f>SUM(modeldata!C12:C15)</f>
@@ -1497,7 +1491,7 @@
         <v>0</v>
       </c>
       <c r="AB6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AC6" s="6">
         <f t="shared" ref="AC6:AC8" si="1">P6-C6</f>
@@ -1546,7 +1540,7 @@
     </row>
     <row r="7" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" s="49">
         <f>SUM('BATS 2023'!P16:P19)</f>
@@ -1593,7 +1587,7 @@
         <v>7901.9660427044219</v>
       </c>
       <c r="O7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P7" s="49">
         <f>SUM(modeldata!C16:C19)</f>
@@ -1640,7 +1634,7 @@
         <v>0</v>
       </c>
       <c r="AB7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AC7" s="8">
         <f t="shared" si="1"/>
@@ -1689,7 +1683,7 @@
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="52">
         <f>SUM(C4:C7)</f>
@@ -1736,7 +1730,7 @@
         <v>986247.94808682636</v>
       </c>
       <c r="O8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P8" s="52">
         <f>SUM(P4:P7)</f>
@@ -1783,7 +1777,7 @@
         <v>0</v>
       </c>
       <c r="AB8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC8">
         <f t="shared" si="1"/>
@@ -1845,7 +1839,7 @@
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" s="43">
         <f>SUM('BATS 2023'!P4,'BATS 2023'!P8,'BATS 2023'!P12,'BATS 2023'!P16)</f>
@@ -1892,7 +1886,7 @@
         <v>773789.05495939124</v>
       </c>
       <c r="O10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P10" s="43">
         <f>modeldata!C4+modeldata!C8+modeldata!C12+modeldata!C16</f>
@@ -1939,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="AB10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AC10" s="3">
         <f>P10-C10</f>
@@ -1988,7 +1982,7 @@
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" s="46">
         <f>SUM('BATS 2023'!P5,'BATS 2023'!P9,'BATS 2023'!P13,'BATS 2023'!P17)</f>
@@ -2035,7 +2029,7 @@
         <v>138952.67010878486</v>
       </c>
       <c r="O11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P11" s="46">
         <f>modeldata!C5+modeldata!C9+modeldata!C13+modeldata!C17</f>
@@ -2082,7 +2076,7 @@
         <v>0</v>
       </c>
       <c r="AB11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AC11" s="6">
         <f>P11-C11</f>
@@ -2131,7 +2125,7 @@
     </row>
     <row r="12" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" s="46">
         <f>SUM('BATS 2023'!P6,'BATS 2023'!P10,'BATS 2023'!P14,'BATS 2023'!P18)</f>
@@ -2178,7 +2172,7 @@
         <v>50928.770542269362</v>
       </c>
       <c r="O12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P12" s="46">
         <f>modeldata!C6+modeldata!C10+modeldata!C14+modeldata!C18</f>
@@ -2225,7 +2219,7 @@
         <v>0</v>
       </c>
       <c r="AB12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AC12" s="6">
         <f t="shared" ref="AC12:AC14" si="33">P12-C12</f>
@@ -2274,7 +2268,7 @@
     </row>
     <row r="13" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" s="49">
         <f>SUM('BATS 2023'!P7,'BATS 2023'!P11,'BATS 2023'!P15,'BATS 2023'!P19)</f>
@@ -2321,7 +2315,7 @@
         <v>22577.452476380953</v>
       </c>
       <c r="O13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P13" s="49">
         <f>modeldata!C7+modeldata!C11+modeldata!C15+modeldata!C19</f>
@@ -2368,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="AB13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AC13" s="8">
         <f t="shared" si="33"/>
@@ -2417,7 +2411,7 @@
     </row>
     <row r="14" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C14" s="52">
         <f>SUM(C10:C13)</f>
@@ -2464,7 +2458,7 @@
         <v>986247.94808682648</v>
       </c>
       <c r="O14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P14" s="52">
         <f>SUM(P10:P13)</f>
@@ -2511,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="AB14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC14">
         <f t="shared" si="33"/>
@@ -2584,7 +2578,7 @@
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="43">
         <f>'BATS 2023'!P4</f>
@@ -2631,7 +2625,7 @@
         <v>675881.93703013682</v>
       </c>
       <c r="O16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P16" s="43">
         <f>modeldata!C4</f>
@@ -2678,7 +2672,7 @@
         <v>0</v>
       </c>
       <c r="AB16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AC16" s="3">
         <f>P16-C16</f>
@@ -2727,7 +2721,7 @@
     </row>
     <row r="17" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" s="46">
         <f>'BATS 2023'!P5+'BATS 2023'!P8</f>
@@ -2774,7 +2768,7 @@
         <v>186753.41224701353</v>
       </c>
       <c r="O17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P17" s="46">
         <f>modeldata!C5+modeldata!C8</f>
@@ -2821,7 +2815,7 @@
         <v>0</v>
       </c>
       <c r="AB17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AC17" s="6">
         <f>P17-C17</f>
@@ -2870,7 +2864,7 @@
     </row>
     <row r="18" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C18" s="46">
         <f>SUM('BATS 2023'!P6,'BATS 2023'!P12,'BATS 2023'!P9)</f>
@@ -2917,7 +2911,7 @@
         <v>72312.696812277689</v>
       </c>
       <c r="O18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P18" s="46">
         <f>modeldata!C6+modeldata!C9+modeldata!C12</f>
@@ -2964,7 +2958,7 @@
         <v>0</v>
       </c>
       <c r="AB18" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="AC18" s="6">
         <f t="shared" ref="AC18:AC20" si="55">P18-C18</f>
@@ -3013,7 +3007,7 @@
     </row>
     <row r="19" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="46">
         <f>SUM('BATS 2023'!P7,'BATS 2023'!P10,'BATS 2023'!P13,'BATS 2023'!P16)</f>
@@ -3060,7 +3054,7 @@
         <v>47050.923678754792</v>
       </c>
       <c r="O19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P19" s="46">
         <f>modeldata!C7+modeldata!C10+modeldata!C13+modeldata!C16</f>
@@ -3107,7 +3101,7 @@
         <v>0</v>
       </c>
       <c r="AB19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AC19" s="6">
         <f t="shared" si="55"/>
@@ -3156,7 +3150,7 @@
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" s="46">
         <f>SUM('BATS 2023'!P11,'BATS 2023'!P14,'BATS 2023'!P17)</f>
@@ -3203,7 +3197,7 @@
         <v>1806.2941002392156</v>
       </c>
       <c r="O20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P20" s="46">
         <f>modeldata!C11+modeldata!C14+modeldata!C17</f>
@@ -3250,7 +3244,7 @@
         <v>0</v>
       </c>
       <c r="AB20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AC20" s="6">
         <f t="shared" si="55"/>
@@ -3299,7 +3293,7 @@
     </row>
     <row r="21" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" s="46">
         <f>SUM('BATS 2023'!P15,'BATS 2023'!P18)</f>
@@ -3346,7 +3340,7 @@
         <v>2442.6842184043094</v>
       </c>
       <c r="O21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P21" s="46">
         <f>modeldata!C15+modeldata!C18</f>
@@ -3393,7 +3387,7 @@
         <v>0</v>
       </c>
       <c r="AB21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AC21" s="6">
         <f>P21-C21</f>
@@ -3442,7 +3436,7 @@
     </row>
     <row r="22" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" s="49">
         <f>'BATS 2023'!P19</f>
@@ -3489,7 +3483,7 @@
         <v>0</v>
       </c>
       <c r="O22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P22" s="49">
         <f>modeldata!C19</f>
@@ -3536,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="AB22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AC22" s="8">
         <f>P22-C22</f>
@@ -3585,7 +3579,7 @@
     </row>
     <row r="23" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" s="52">
         <f>SUM(C16:C22)</f>
@@ -3632,7 +3626,7 @@
         <v>986247.94808682636</v>
       </c>
       <c r="O23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P23" s="52">
         <f>SUM(P16:P22)</f>
@@ -3679,7 +3673,7 @@
         <v>0</v>
       </c>
       <c r="AB23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC23">
         <f t="shared" ref="AC23" si="77">P23-C23</f>
@@ -3729,7 +3723,7 @@
     <row r="25" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A25" s="12"/>
       <c r="B25" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="12"/>
       <c r="D25" s="12"/>
@@ -3744,7 +3738,7 @@
       <c r="M25" s="12"/>
       <c r="N25" s="12"/>
       <c r="O25" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P25" s="12"/>
       <c r="Q25" s="12"/>
@@ -3759,7 +3753,7 @@
       <c r="Z25" s="12"/>
       <c r="AA25" s="12"/>
       <c r="AB25" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AC25" s="12"/>
       <c r="AD25" s="12"/>
@@ -3876,7 +3870,7 @@
     </row>
     <row r="27" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" s="53">
         <f t="shared" ref="C27:M27" si="78">C4/C$8</f>
@@ -3923,7 +3917,7 @@
         <v>0.8682853920727599</v>
       </c>
       <c r="O27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P27" s="64" t="e">
         <f>P4/P$8</f>
@@ -3970,7 +3964,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AC27" s="64" t="e">
         <f>P27-C27</f>
@@ -4019,7 +4013,7 @@
     </row>
     <row r="28" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" s="56">
         <f t="shared" ref="C28:M28" si="90">C5/C$8</f>
@@ -4066,7 +4060,7 @@
         <v>8.5456080319816399E-2</v>
       </c>
       <c r="O28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P28" s="67" t="e">
         <f t="shared" ref="P28:P30" si="91">P5/P$8</f>
@@ -4113,7 +4107,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AC28" s="67" t="e">
         <f>P28-C28</f>
@@ -4162,7 +4156,7 @@
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C29" s="56">
         <f t="shared" ref="C29:M29" si="93">C6/C$8</f>
@@ -4209,7 +4203,7 @@
         <v>3.824637806832145E-2</v>
       </c>
       <c r="O29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P29" s="67" t="e">
         <f t="shared" si="91"/>
@@ -4256,7 +4250,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AC29" s="67" t="e">
         <f t="shared" ref="AC29:AC31" si="95">P29-C29</f>
@@ -4305,7 +4299,7 @@
     </row>
     <row r="30" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" s="59">
         <f t="shared" ref="C30:M30" si="96">C7/C$8</f>
@@ -4352,7 +4346,7 @@
         <v>8.012149539102266E-3</v>
       </c>
       <c r="O30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P30" s="70" t="e">
         <f t="shared" si="91"/>
@@ -4399,7 +4393,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AC30" s="70" t="e">
         <f t="shared" si="95"/>
@@ -4448,7 +4442,7 @@
     </row>
     <row r="31" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C31" s="62">
         <f t="shared" ref="C31:M31" si="98">C8/C$8</f>
@@ -4495,7 +4489,7 @@
         <v>1</v>
       </c>
       <c r="O31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P31" s="68" t="e">
         <f>P8/P$8</f>
@@ -4542,7 +4536,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC31" s="68" t="e">
         <f t="shared" si="95"/>
@@ -4626,7 +4620,7 @@
     </row>
     <row r="33" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" s="53">
         <f t="shared" ref="C33:M33" si="100">C10/C$14</f>
@@ -4673,7 +4667,7 @@
         <v>0.78457862088375063</v>
       </c>
       <c r="O33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P33" s="64" t="e">
         <f>P10/P$14</f>
@@ -4720,7 +4714,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AC33" s="64" t="e">
         <f>P33-C33</f>
@@ -4769,7 +4763,7 @@
     </row>
     <row r="34" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C34" s="56">
         <f t="shared" ref="C34:M34" si="112">C11/C$14</f>
@@ -4816,7 +4810,7 @@
         <v>0.14089019944561837</v>
       </c>
       <c r="O34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P34" s="67" t="e">
         <f t="shared" ref="P34:P36" si="113">P11/P$14</f>
@@ -4863,7 +4857,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AC34" s="67" t="e">
         <f>P34-C34</f>
@@ -4912,7 +4906,7 @@
     </row>
     <row r="35" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" s="56">
         <f t="shared" ref="C35:M35" si="115">C12/C$14</f>
@@ -4959,7 +4953,7 @@
         <v>5.1638911534430627E-2</v>
       </c>
       <c r="O35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P35" s="67" t="e">
         <f t="shared" si="113"/>
@@ -5006,7 +5000,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AC35" s="67" t="e">
         <f t="shared" ref="AC35:AC37" si="117">P35-C35</f>
@@ -5055,7 +5049,7 @@
     </row>
     <row r="36" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" s="59">
         <f t="shared" ref="C36:M36" si="118">C13/C$14</f>
@@ -5102,7 +5096,7 @@
         <v>2.2892268136200267E-2</v>
       </c>
       <c r="O36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P36" s="70" t="e">
         <f t="shared" si="113"/>
@@ -5149,7 +5143,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AC36" s="70" t="e">
         <f t="shared" si="117"/>
@@ -5198,7 +5192,7 @@
     </row>
     <row r="37" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C37" s="62">
         <f t="shared" ref="C37:M37" si="120">C14/C$14</f>
@@ -5245,7 +5239,7 @@
         <v>1</v>
       </c>
       <c r="O37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P37" s="68" t="e">
         <f>P14/P$14</f>
@@ -5292,7 +5286,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC37" s="68" t="e">
         <f t="shared" si="117"/>
@@ -5376,7 +5370,7 @@
     </row>
     <row r="39" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C39" s="53">
         <f t="shared" ref="C39:M39" si="122">C16/C$23</f>
@@ -5423,7 +5417,7 @@
         <v>0.68530630491170785</v>
       </c>
       <c r="O39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P39" s="64" t="e">
         <f>P16/P$23</f>
@@ -5470,7 +5464,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB39" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AC39" s="64" t="e">
         <f>P39-C39</f>
@@ -5519,7 +5513,7 @@
     </row>
     <row r="40" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C40" s="56">
         <f t="shared" ref="C40:M40" si="134">C17/C$23</f>
@@ -5566,7 +5560,7 @@
         <v>0.18935746594888966</v>
       </c>
       <c r="O40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P40" s="67" t="e">
         <f t="shared" ref="P40:P45" si="135">P17/P$23</f>
@@ -5613,7 +5607,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AC40" s="67" t="e">
         <f>P40-C40</f>
@@ -5662,7 +5656,7 @@
     </row>
     <row r="41" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C41" s="56">
         <f t="shared" ref="C41:M41" si="137">C18/C$23</f>
@@ -5709,7 +5703,7 @@
         <v>7.3321011164133226E-2</v>
       </c>
       <c r="O41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P41" s="67" t="e">
         <f t="shared" si="135"/>
@@ -5756,7 +5750,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="AC41" s="67" t="e">
         <f t="shared" ref="AC41:AC43" si="139">P41-C41</f>
@@ -5805,7 +5799,7 @@
     </row>
     <row r="42" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C42" s="56">
         <f t="shared" ref="C42:M42" si="140">C19/C$23</f>
@@ -5852,7 +5846,7 @@
         <v>4.7706992719251336E-2</v>
       </c>
       <c r="O42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P42" s="67" t="e">
         <f t="shared" si="135"/>
@@ -5899,7 +5893,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AC42" s="67" t="e">
         <f t="shared" si="139"/>
@@ -5948,7 +5942,7 @@
     </row>
     <row r="43" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C43" s="56">
         <f t="shared" ref="C43:M43" si="142">C20/C$23</f>
@@ -5995,7 +5989,7 @@
         <v>1.8314807181532354E-3</v>
       </c>
       <c r="O43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P43" s="67" t="e">
         <f t="shared" si="135"/>
@@ -6042,7 +6036,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AC43" s="67" t="e">
         <f t="shared" si="139"/>
@@ -6091,7 +6085,7 @@
     </row>
     <row r="44" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C44" s="56">
         <f t="shared" ref="C44:M44" si="144">C21/C$23</f>
@@ -6138,7 +6132,7 @@
         <v>2.4767445378646941E-3</v>
       </c>
       <c r="O44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P44" s="67" t="e">
         <f t="shared" si="135"/>
@@ -6185,7 +6179,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AC44" s="67" t="e">
         <f>P44-C44</f>
@@ -6234,7 +6228,7 @@
     </row>
     <row r="45" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C45" s="59">
         <f t="shared" ref="C45:M45" si="146">C22/C$23</f>
@@ -6281,7 +6275,7 @@
         <v>0</v>
       </c>
       <c r="O45" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P45" s="70" t="e">
         <f t="shared" si="135"/>
@@ -6328,7 +6322,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB45" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AC45" s="70" t="e">
         <f>P45-C45</f>
@@ -6377,7 +6371,7 @@
     </row>
     <row r="46" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C46" s="62">
         <f t="shared" ref="C46:M46" si="148">C23/C$23</f>
@@ -6424,7 +6418,7 @@
         <v>1</v>
       </c>
       <c r="O46" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P46" s="68" t="e">
         <f>P23/P$23</f>
@@ -6471,7 +6465,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB46" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC46" s="68" t="e">
         <f t="shared" ref="AC46" si="150">P46-C46</f>
@@ -6520,19 +6514,19 @@
     </row>
     <row r="48" spans="2:39" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C48" s="11"/>
     </row>
     <row r="50" spans="1:39" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
+        <v>50</v>
+      </c>
+      <c r="O50" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB50" t="s">
         <v>51</v>
-      </c>
-      <c r="O50" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB50" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:39" x14ac:dyDescent="0.25">
@@ -6638,10 +6632,10 @@
     </row>
     <row r="52" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B52" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C52" s="16" cm="1">
         <f t="array" ref="C52">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A52),0),MATCH(calibration!$B52,constants!$C$4:$R$4,0))</f>
@@ -6688,7 +6682,7 @@
         <v>0</v>
       </c>
       <c r="O52" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P52" s="16" t="e">
         <f>$C$48*LN(C27/P27)</f>
@@ -6735,7 +6729,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB52" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="AC52" s="16"/>
       <c r="AD52" s="17"/>
@@ -6751,10 +6745,10 @@
     </row>
     <row r="53" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C53" s="19" cm="1">
         <f t="array" ref="C53">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A53),0),MATCH(calibration!$B53,constants!$C$4:$R$4,0))</f>
@@ -6801,7 +6795,7 @@
         <v>0</v>
       </c>
       <c r="O53" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="P53" s="19" t="e">
         <f>$C$48*LN(C28/P28)</f>
@@ -6848,7 +6842,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB53" s="15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AC53" s="19" t="e">
         <f>C53+P53-$P$52</f>
@@ -6897,10 +6891,10 @@
     </row>
     <row r="54" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B54" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C54" s="19" cm="1">
         <f t="array" ref="C54">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A54),0),MATCH(calibration!$B54,constants!$C$4:$R$4,0))</f>
@@ -6947,7 +6941,7 @@
         <v>0</v>
       </c>
       <c r="O54" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="P54" s="19" t="e">
         <f>$C$48*LN(C29/P29)</f>
@@ -6994,7 +6988,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB54" s="15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AC54" s="19" t="e">
         <f t="shared" ref="AC54:AC55" si="155">C54+P54-$P$52</f>
@@ -7043,10 +7037,10 @@
     </row>
     <row r="55" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B55" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C55" s="21" cm="1">
         <f t="array" ref="C55">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A55),0),MATCH(calibration!$B55,constants!$C$4:$R$4,0))</f>
@@ -7093,7 +7087,7 @@
         <v>0</v>
       </c>
       <c r="O55" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P55" s="21" t="e">
         <f>$C$48*LN(C30/P30)</f>
@@ -7140,7 +7134,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB55" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AC55" s="19" t="e">
         <f t="shared" si="155"/>
@@ -7189,10 +7183,10 @@
     </row>
     <row r="56" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C56" s="24" cm="1">
         <f t="array" ref="C56">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A56),0),MATCH(calibration!$B56,constants!$C$5:$R$5,0))</f>
@@ -7239,7 +7233,7 @@
         <v>0</v>
       </c>
       <c r="O56" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P56" s="24" t="e">
         <f>$C$48*LN(C33/P33)</f>
@@ -7286,7 +7280,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB56" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AC56" s="24"/>
       <c r="AD56" s="25"/>
@@ -7302,10 +7296,10 @@
     </row>
     <row r="57" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C57" s="27" cm="1">
         <f t="array" ref="C57">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A57),0),MATCH(calibration!$B57,constants!$C$5:$R$5,0))</f>
@@ -7352,7 +7346,7 @@
         <v>0</v>
       </c>
       <c r="O57" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P57" s="27" t="e">
         <f>$C$48*LN(C34/P34)</f>
@@ -7399,7 +7393,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB57" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AC57" s="27" t="e">
         <f t="shared" ref="AC57:AC58" si="159">C57+P57-$P$52</f>
@@ -7448,10 +7442,10 @@
     </row>
     <row r="58" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C58" s="27" cm="1">
         <f t="array" ref="C58">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A58),0),MATCH(calibration!$B58,constants!$C$5:$R$5,0))</f>
@@ -7498,7 +7492,7 @@
         <v>0</v>
       </c>
       <c r="O58" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P58" s="27" t="e">
         <f>$C$48*LN(C35/P35)</f>
@@ -7545,7 +7539,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB58" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="AC58" s="27" t="e">
         <f t="shared" si="159"/>
@@ -7594,10 +7588,10 @@
     </row>
     <row r="59" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C59" s="29" cm="1">
         <f t="array" ref="C59">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A59),0),MATCH(calibration!$B59,constants!$C$5:$R$5,0))</f>
@@ -7644,7 +7638,7 @@
         <v>0</v>
       </c>
       <c r="O59" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P59" s="29" t="e">
         <f>$C$48*LN(C36/P36)</f>
@@ -7691,7 +7685,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB59" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AC59" s="29" t="e">
         <f t="shared" ref="AC59" si="171">C59+P59-$P$52</f>
@@ -7740,10 +7734,10 @@
     </row>
     <row r="60" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B60" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C60" s="32" cm="1">
         <f t="array" ref="C60">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A60),0),MATCH(calibration!$B60,constants!$C$3:$R$3,0))</f>
@@ -7790,7 +7784,7 @@
         <v>0</v>
       </c>
       <c r="O60" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="P60" s="32" t="e">
         <f t="shared" ref="P60:P66" si="181">$C$48*LN(C39/P39)</f>
@@ -7837,7 +7831,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB60" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AC60" s="32"/>
       <c r="AD60" s="33"/>
@@ -7853,10 +7847,10 @@
     </row>
     <row r="61" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C61" s="35" cm="1">
         <f t="array" ref="C61">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A61),0),MATCH(calibration!$B61,constants!$C$3:$R$3,0))</f>
@@ -7903,7 +7897,7 @@
         <v>0</v>
       </c>
       <c r="O61" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="P61" s="35" t="e">
         <f t="shared" si="181"/>
@@ -7950,7 +7944,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB61" s="14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="AC61" s="35"/>
       <c r="AD61" s="14"/>
@@ -7966,10 +7960,10 @@
     </row>
     <row r="62" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B62" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C62" s="35" cm="1">
         <f t="array" ref="C62">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A62),0),MATCH(calibration!$B62,constants!$C$3:$R$3,0))</f>
@@ -8016,7 +8010,7 @@
         <v>0</v>
       </c>
       <c r="O62" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P62" s="35" t="e">
         <f t="shared" si="181"/>
@@ -8063,7 +8057,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB62" s="14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="AC62" s="35" t="e">
         <f t="shared" ref="AC62:AC66" si="185">C62+P62-$P$60</f>
@@ -8112,10 +8106,10 @@
     </row>
     <row r="63" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C63" s="35" cm="1">
         <f t="array" ref="C63">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A63),0),MATCH(calibration!$B63,constants!$C$3:$R$3,0))</f>
@@ -8162,7 +8156,7 @@
         <v>0</v>
       </c>
       <c r="O63" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="P63" s="35" t="e">
         <f t="shared" si="181"/>
@@ -8209,7 +8203,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB63" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AC63" s="35" t="e">
         <f t="shared" si="185"/>
@@ -8258,10 +8252,10 @@
     </row>
     <row r="64" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B64" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C64" s="35" cm="1">
         <f t="array" ref="C64">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A64),0),MATCH(calibration!$B64,constants!$C$3:$R$3,0))</f>
@@ -8308,7 +8302,7 @@
         <v>0</v>
       </c>
       <c r="O64" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="P64" s="35" t="e">
         <f t="shared" si="181"/>
@@ -8355,7 +8349,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB64" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AC64" s="35" t="e">
         <f t="shared" si="185"/>
@@ -8404,10 +8398,10 @@
     </row>
     <row r="65" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B65" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C65" s="35" cm="1">
         <f t="array" ref="C65">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A65),0),MATCH(calibration!$B65,constants!$C$3:$R$3,0))</f>
@@ -8454,7 +8448,7 @@
         <v>0</v>
       </c>
       <c r="O65" s="14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P65" s="35" t="e">
         <f t="shared" si="181"/>
@@ -8501,7 +8495,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB65" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AC65" s="35" t="e">
         <f t="shared" si="185"/>
@@ -8550,10 +8544,10 @@
     </row>
     <row r="66" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B66" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C66" s="37" cm="1">
         <f t="array" ref="C66">INDEX(constants!$C$6:$R$38,MATCH(1,(constants!$A$6:$A$38=calibration!C$51)*(constants!$B$6:$B$38=calibration!$A66),0),MATCH(calibration!$B66,constants!$C$3:$R$3,0))</f>
@@ -8600,7 +8594,7 @@
         <v>0</v>
       </c>
       <c r="O66" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P66" s="37" t="e">
         <f t="shared" si="181"/>
@@ -8647,7 +8641,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="AB66" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AC66" s="37" t="e">
         <f t="shared" si="185"/>
@@ -8696,7 +8690,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="AC27:AM45">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>ABS(AC27) &gt; 10%</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8714,405 +8708,405 @@
   <sheetData>
     <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="C1" s="73" t="s">
+        <v>84</v>
+      </c>
+      <c r="S1" s="73" t="s">
         <v>85</v>
-      </c>
-      <c r="S1" s="73" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" t="s">
         <v>63</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>64</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>65</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>66</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>67</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>68</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>69</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>70</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>71</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>72</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>73</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>74</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>75</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>76</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="R2" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="S2" t="s">
+        <v>62</v>
+      </c>
+      <c r="T2" t="s">
         <v>63</v>
       </c>
-      <c r="T2" t="s">
+      <c r="U2" t="s">
         <v>64</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" t="s">
         <v>65</v>
       </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>66</v>
       </c>
-      <c r="W2" t="s">
+      <c r="X2" t="s">
         <v>67</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Y2" t="s">
         <v>68</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>69</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>70</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>71</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>72</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>73</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>74</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AF2" t="s">
         <v>75</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="AG2" t="s">
         <v>76</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AH2" t="s">
         <v>77</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s">
         <v>37</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>38</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" t="s">
+        <v>78</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" t="s">
+        <v>78</v>
+      </c>
+      <c r="N3" t="s">
+        <v>79</v>
+      </c>
+      <c r="O3" t="s">
+        <v>38</v>
+      </c>
+      <c r="P3" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>79</v>
+      </c>
+      <c r="R3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G3" t="s">
+      <c r="S3" t="s">
+        <v>42</v>
+      </c>
+      <c r="T3" t="s">
+        <v>36</v>
+      </c>
+      <c r="U3" t="s">
         <v>37</v>
       </c>
-      <c r="H3" t="s">
+      <c r="V3" t="s">
         <v>38</v>
       </c>
-      <c r="I3" t="s">
+      <c r="W3" t="s">
+        <v>36</v>
+      </c>
+      <c r="X3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AH3" t="s">
         <v>39</v>
-      </c>
-      <c r="J3" t="s">
-        <v>79</v>
-      </c>
-      <c r="K3" t="s">
-        <v>38</v>
-      </c>
-      <c r="L3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" t="s">
-        <v>79</v>
-      </c>
-      <c r="N3" t="s">
-        <v>80</v>
-      </c>
-      <c r="O3" t="s">
-        <v>39</v>
-      </c>
-      <c r="P3" t="s">
-        <v>79</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>80</v>
-      </c>
-      <c r="R3" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="S3" t="s">
-        <v>43</v>
-      </c>
-      <c r="T3" t="s">
-        <v>37</v>
-      </c>
-      <c r="U3" t="s">
-        <v>38</v>
-      </c>
-      <c r="V3" t="s">
-        <v>39</v>
-      </c>
-      <c r="W3" t="s">
-        <v>37</v>
-      </c>
-      <c r="X3" t="s">
-        <v>38</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>39</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AF3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AG3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
         <v>33</v>
       </c>
-      <c r="D4" t="s">
+      <c r="H4" t="s">
         <v>33</v>
       </c>
-      <c r="E4" t="s">
+      <c r="I4" t="s">
         <v>33</v>
       </c>
-      <c r="F4" t="s">
+      <c r="J4" t="s">
         <v>33</v>
       </c>
-      <c r="G4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" t="s">
-        <v>34</v>
-      </c>
-      <c r="J4" t="s">
-        <v>34</v>
-      </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="M4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S4" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" t="s">
+        <v>32</v>
+      </c>
+      <c r="U4" t="s">
+        <v>32</v>
+      </c>
+      <c r="V4" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4" t="s">
         <v>33</v>
       </c>
-      <c r="T4" t="s">
+      <c r="X4" t="s">
         <v>33</v>
       </c>
-      <c r="U4" t="s">
+      <c r="Y4" t="s">
         <v>33</v>
       </c>
-      <c r="V4" t="s">
+      <c r="Z4" t="s">
         <v>33</v>
       </c>
-      <c r="W4" t="s">
-        <v>34</v>
-      </c>
-      <c r="X4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>34</v>
-      </c>
       <c r="AA4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AB4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AC4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AD4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AE4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AF4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AG4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="AH4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A5" s="73" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="G5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="H5" s="9" t="s">
+      <c r="I5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="9" t="s">
+      <c r="J5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="K5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="9" t="s">
+      <c r="M5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="M5" s="9" t="s">
+      <c r="N5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="N5" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="O5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="P5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="Q5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="R5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="R5" s="10" t="s">
-        <v>32</v>
-      </c>
       <c r="S5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="T5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="T5" s="9" t="s">
+      <c r="U5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="U5" s="9" t="s">
+      <c r="V5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="V5" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="W5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="X5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="X5" s="9" t="s">
+      <c r="Y5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="Y5" s="9" t="s">
+      <c r="Z5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="Z5" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="AA5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AB5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="AB5" s="9" t="s">
+      <c r="AC5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="AC5" s="9" t="s">
+      <c r="AD5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="AD5" s="9" t="s">
-        <v>32</v>
-      </c>
       <c r="AE5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="AF5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="AF5" s="9" t="s">
+      <c r="AG5" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="AG5" s="9" t="s">
+      <c r="AH5" s="9" t="s">
         <v>31</v>
-      </c>
-      <c r="AH5" s="9" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
@@ -9120,7 +9114,7 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R6" s="7"/>
       <c r="S6">
@@ -9193,7 +9187,7 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R7" s="7"/>
       <c r="S7">
@@ -9266,7 +9260,7 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R8" s="7"/>
       <c r="S8">
@@ -9339,7 +9333,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R9" s="7"/>
       <c r="S9">
@@ -9412,7 +9406,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R10" s="7"/>
       <c r="S10">
@@ -9485,7 +9479,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R11" s="7"/>
       <c r="S11">
@@ -9558,7 +9552,7 @@
         <v>3</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R12" s="7"/>
       <c r="S12">
@@ -9631,7 +9625,7 @@
         <v>3</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R13" s="7"/>
       <c r="S13">
@@ -9704,7 +9698,7 @@
         <v>3</v>
       </c>
       <c r="B14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R14" s="7"/>
       <c r="S14">
@@ -9777,7 +9771,7 @@
         <v>4</v>
       </c>
       <c r="B15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R15" s="7"/>
       <c r="S15">
@@ -9850,7 +9844,7 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R16" s="7"/>
       <c r="S16">
@@ -9923,7 +9917,7 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R17" s="7"/>
       <c r="S17">
@@ -9996,7 +9990,7 @@
         <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R18" s="7"/>
       <c r="S18">
@@ -10069,7 +10063,7 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R19" s="7"/>
       <c r="S19">
@@ -10142,7 +10136,7 @@
         <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R20" s="7"/>
       <c r="S20">
@@ -10215,7 +10209,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R21" s="7"/>
       <c r="S21">
@@ -10288,7 +10282,7 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R22" s="7"/>
       <c r="S22">
@@ -10361,7 +10355,7 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R23" s="7"/>
       <c r="S23">
@@ -10434,7 +10428,7 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R24" s="7"/>
       <c r="S24">
@@ -10507,7 +10501,7 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R25" s="7"/>
       <c r="S25">
@@ -10580,7 +10574,7 @@
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R26" s="7"/>
       <c r="S26">
@@ -10653,7 +10647,7 @@
         <v>8</v>
       </c>
       <c r="B27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R27" s="7"/>
       <c r="S27">
@@ -10726,7 +10720,7 @@
         <v>8</v>
       </c>
       <c r="B28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R28" s="7"/>
       <c r="S28">
@@ -10799,7 +10793,7 @@
         <v>8</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R29" s="7"/>
       <c r="S29">
@@ -10872,7 +10866,7 @@
         <v>9</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R30" s="7"/>
       <c r="S30">
@@ -10945,7 +10939,7 @@
         <v>9</v>
       </c>
       <c r="B31" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R31" s="7"/>
       <c r="S31">
@@ -11018,7 +11012,7 @@
         <v>9</v>
       </c>
       <c r="B32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R32" s="7"/>
       <c r="S32">
@@ -11091,7 +11085,7 @@
         <v>10</v>
       </c>
       <c r="B33" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R33" s="7"/>
       <c r="S33">
@@ -11164,7 +11158,7 @@
         <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R34" s="7"/>
       <c r="S34">
@@ -11237,7 +11231,7 @@
         <v>10</v>
       </c>
       <c r="B35" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R35" s="7"/>
       <c r="S35">
@@ -11310,7 +11304,7 @@
         <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R36" s="7"/>
       <c r="S36">
@@ -11383,7 +11377,7 @@
         <v>11</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R37" s="7"/>
       <c r="S37">
@@ -11456,7 +11450,7 @@
         <v>11</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R38" s="7"/>
       <c r="S38">
@@ -11700,7 +11694,7 @@
   <sheetData>
     <row r="1" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="2:26" x14ac:dyDescent="0.25">
@@ -12113,7 +12107,7 @@
     </row>
     <row r="8" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" s="42">
         <v>25474.951198525359</v>
@@ -12529,7 +12523,7 @@
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C13" s="42">
         <v>15059.392755897852</v>
@@ -12932,7 +12926,7 @@
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C18" s="42">
         <v>12594.924073455264</v>
@@ -13180,7 +13174,7 @@
     </row>
     <row r="23" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C23" s="42">
         <v>1668.63177660064</v>
@@ -13208,7 +13202,7 @@
     </row>
     <row r="24" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C24" s="42">
         <v>16199.986463378213</v>
@@ -13244,7 +13238,7 @@
     </row>
     <row r="25" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C25" s="42">
         <v>15058.072609072527</v>
@@ -13274,7 +13268,7 @@
     </row>
     <row r="26" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="42">
         <v>12989.715378425308</v>
@@ -13304,7 +13298,7 @@
     </row>
     <row r="27" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C27" s="42">
         <v>765.92383367125706</v>
@@ -13334,7 +13328,7 @@
     </row>
     <row r="28" spans="2:26" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28" s="42">
         <v>6877.3667650190509</v>

</xml_diff>